<commit_message>
Mise à jour du portfolio et des documents BTS
</commit_message>
<xml_diff>
--- a/DOSSIER A INTEGRER/Tableau_de_synthese_-_Epreuve_E5_-_BTS_SIO_REBECCA_BOSAKE.xlsx
+++ b/DOSSIER A INTEGRER/Tableau_de_synthese_-_Epreuve_E5_-_BTS_SIO_REBECCA_BOSAKE.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.bosake\Downloads\portfolio-becky - PRESENTATION_OFFICIEL\DOSSIER A INTEGRER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1620F60F-65CD-4E34-A029-0466C4FB8E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBF5CDE-2DCC-4563-98BF-7AF5165FAEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="624" yWindow="624" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$39</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>2025-2026</t>
+  </si>
+  <si>
+    <t>URL du site :https://bzuena27.github.io/</t>
   </si>
 </sst>
 </file>
@@ -571,7 +574,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -649,15 +652,33 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -681,15 +702,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -999,7 +1011,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ84"/>
+  <dimension ref="A1:AQ85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -1010,160 +1022,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="29"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="38" t="s">
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="39"/>
-      <c r="H3" s="40"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="33"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+    <row r="4" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="9" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" spans="1:43" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H5" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B6" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.35000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="20" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.35000000000002" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="35"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H7" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6"/>
-      <c r="M6"/>
-      <c r="N6"/>
-      <c r="O6"/>
-      <c r="P6"/>
-      <c r="Q6"/>
-      <c r="R6"/>
-      <c r="S6"/>
-      <c r="T6"/>
-      <c r="U6"/>
-      <c r="V6"/>
-      <c r="W6"/>
-      <c r="X6"/>
-      <c r="Y6"/>
-      <c r="Z6"/>
-      <c r="AA6"/>
-      <c r="AB6"/>
-      <c r="AC6"/>
-      <c r="AD6"/>
-      <c r="AE6"/>
-      <c r="AF6"/>
-      <c r="AG6"/>
-      <c r="AH6"/>
-      <c r="AI6"/>
-      <c r="AJ6"/>
-      <c r="AK6"/>
-      <c r="AL6"/>
-      <c r="AM6"/>
-      <c r="AN6"/>
-      <c r="AO6"/>
-      <c r="AP6"/>
-      <c r="AQ6"/>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="32"/>
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
@@ -1201,14 +1181,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
+      <c r="A8" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1245,19 +1227,15 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="13"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A9" s="14"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1296,16 +1274,16 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="23"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="12"/>
       <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="12"/>
       <c r="H10" s="13"/>
       <c r="I10"/>
       <c r="J10"/>
@@ -1345,16 +1323,16 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
+      <c r="D11" s="12"/>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="G11" s="23"/>
       <c r="H11" s="13"/>
       <c r="I11"/>
       <c r="J11"/>
@@ -1394,12 +1372,12 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="12"/>
+      <c r="C12" s="23"/>
       <c r="D12" s="23"/>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
@@ -1443,16 +1421,16 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="23"/>
+      <c r="G13" s="12"/>
       <c r="H13" s="13"/>
       <c r="I13"/>
       <c r="J13"/>
@@ -1492,16 +1470,16 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="23"/>
+      <c r="C14" s="12"/>
       <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="12"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="23"/>
       <c r="H14" s="13"/>
       <c r="I14"/>
       <c r="J14"/>
@@ -1541,16 +1519,16 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="12"/>
+      <c r="C15" s="23"/>
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="12"/>
       <c r="H15" s="13"/>
       <c r="I15"/>
       <c r="J15"/>
@@ -1590,15 +1568,15 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C16" s="12"/>
-      <c r="D16" s="23"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="23"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="23"/>
       <c r="H16" s="13"/>
       <c r="I16"/>
@@ -1639,15 +1617,15 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
+      <c r="D17" s="23"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
+      <c r="F17" s="23"/>
       <c r="G17" s="23"/>
       <c r="H17" s="13"/>
       <c r="I17"/>
@@ -1688,16 +1666,16 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
-      <c r="E18" s="23"/>
+      <c r="E18" s="12"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="G18" s="23"/>
       <c r="H18" s="13"/>
       <c r="I18"/>
       <c r="J18"/>
@@ -1737,17 +1715,17 @@
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+      <c r="E19" s="23"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
-      <c r="H19" s="24"/>
+      <c r="H19" s="13"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1786,7 +1764,7 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="26" t="s">
         <v>52</v>
@@ -1795,8 +1773,8 @@
       <c r="D20" s="12"/>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="13"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="24"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1835,16 +1813,16 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="23"/>
+      <c r="C21" s="12"/>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
+      <c r="G21" s="23"/>
       <c r="H21" s="13"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -1884,17 +1862,17 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="12"/>
+      <c r="C22" s="23"/>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
-      <c r="H22" s="24"/>
+      <c r="H22" s="13"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1933,7 +1911,7 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" s="26" t="s">
         <v>52</v>
@@ -1941,9 +1919,9 @@
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
       <c r="E23" s="12"/>
-      <c r="F23" s="23"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="12"/>
-      <c r="H23" s="13"/>
+      <c r="H23" s="24"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1980,17 +1958,19 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="35"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="13"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2027,19 +2007,17 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B25" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="13"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A25" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="41"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2078,17 +2056,17 @@
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B26" s="26" t="s">
         <v>53</v>
       </c>
       <c r="C26" s="23"/>
       <c r="D26" s="23"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
       <c r="G26" s="23"/>
-      <c r="H26" s="19"/>
+      <c r="H26" s="13"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2127,7 +2105,7 @@
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="26" t="s">
         <v>53</v>
@@ -2176,16 +2154,16 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B28" s="26" t="s">
         <v>53</v>
       </c>
       <c r="C28" s="23"/>
-      <c r="D28" s="18"/>
+      <c r="D28" s="23"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
+      <c r="G28" s="23"/>
       <c r="H28" s="19"/>
       <c r="I28"/>
       <c r="J28"/>
@@ -2225,16 +2203,16 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B29" s="26" t="s">
         <v>53</v>
       </c>
       <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
+      <c r="D29" s="18"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
-      <c r="G29" s="23"/>
+      <c r="G29" s="18"/>
       <c r="H29" s="19"/>
       <c r="I29"/>
       <c r="J29"/>
@@ -2272,17 +2250,19 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A30" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="35"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="19"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2319,20 +2299,18 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="25"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A31" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="40"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="41"/>
+      <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
       <c r="L31"/>
@@ -2370,17 +2348,17 @@
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C32" s="23"/>
       <c r="D32" s="23"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
       <c r="G32" s="23"/>
-      <c r="H32" s="19"/>
+      <c r="H32" s="13"/>
       <c r="I32" s="25"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2419,18 +2397,18 @@
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B33" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C33" s="23"/>
       <c r="D33" s="23"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="23"/>
-      <c r="H33" s="13"/>
-      <c r="I33"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="25"/>
       <c r="J33"/>
       <c r="K33"/>
       <c r="L33"/>
@@ -2468,16 +2446,16 @@
     </row>
     <row r="34" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B34" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C34" s="23"/>
-      <c r="D34" s="12"/>
+      <c r="D34" s="23"/>
       <c r="E34" s="12"/>
       <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
+      <c r="G34" s="23"/>
       <c r="H34" s="13"/>
       <c r="I34"/>
       <c r="J34"/>
@@ -2517,16 +2495,16 @@
     </row>
     <row r="35" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B35" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
+      <c r="D35" s="12"/>
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
-      <c r="G35" s="23"/>
+      <c r="G35" s="12"/>
       <c r="H35" s="13"/>
       <c r="I35"/>
       <c r="J35"/>
@@ -2566,7 +2544,7 @@
     </row>
     <row r="36" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B36" s="26" t="s">
         <v>52</v>
@@ -2615,16 +2593,16 @@
     </row>
     <row r="37" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B37" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C37" s="23"/>
-      <c r="D37" s="12"/>
+      <c r="D37" s="23"/>
       <c r="E37" s="12"/>
       <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
+      <c r="G37" s="23"/>
       <c r="H37" s="13"/>
       <c r="I37"/>
       <c r="J37"/>
@@ -2662,15 +2640,19 @@
       <c r="AP37"/>
       <c r="AQ37"/>
     </row>
-    <row r="38" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A38" s="5"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+    <row r="38" spans="1:43" s="2" customFormat="1" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="23"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="13"/>
       <c r="I38"/>
       <c r="J38"/>
       <c r="K38"/>
@@ -2707,7 +2689,51 @@
       <c r="AP38"/>
       <c r="AQ38"/>
     </row>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A39" s="5"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+      <c r="L39"/>
+      <c r="M39"/>
+      <c r="N39"/>
+      <c r="O39"/>
+      <c r="P39"/>
+      <c r="Q39"/>
+      <c r="R39"/>
+      <c r="S39"/>
+      <c r="T39"/>
+      <c r="U39"/>
+      <c r="V39"/>
+      <c r="W39"/>
+      <c r="X39"/>
+      <c r="Y39"/>
+      <c r="Z39"/>
+      <c r="AA39"/>
+      <c r="AB39"/>
+      <c r="AC39"/>
+      <c r="AD39"/>
+      <c r="AE39"/>
+      <c r="AF39"/>
+      <c r="AG39"/>
+      <c r="AH39"/>
+      <c r="AI39"/>
+      <c r="AJ39"/>
+      <c r="AK39"/>
+      <c r="AL39"/>
+      <c r="AM39"/>
+      <c r="AN39"/>
+      <c r="AO39"/>
+      <c r="AP39"/>
+      <c r="AQ39"/>
+    </row>
     <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2745,31 +2771,33 @@
     <row r="74" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="75" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77">
+    <row r="77" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="80" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="84" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="85" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A4:E4"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2780,6 +2808,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010021F07685AB1D6D42B1C8754387C28D03" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="db6b390132c6309ae4cfd2628f9bb9bf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4d1d7550-f116-4197-9c89-6add1d81ee4d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9af7643d011b158d68af97117a02b1a" ns2:_="">
     <xsd:import namespace="4d1d7550-f116-4197-9c89-6add1d81ee4d"/>
@@ -2941,22 +2984,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{157607A9-BAFB-45F5-9C7F-B4070279AD02}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="4d1d7550-f116-4197-9c89-6add1d81ee4d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70D8B243-4BAE-4BAD-AD28-E1C4834C0A4E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B192E8B-391C-4855-A857-911639F4CCBE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2974,30 +3026,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70D8B243-4BAE-4BAD-AD28-E1C4834C0A4E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{157607A9-BAFB-45F5-9C7F-B4070279AD02}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="4d1d7550-f116-4197-9c89-6add1d81ee4d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{dfdd9a14-7b84-416b-97e8-b834b0f98713}" enabled="1" method="Standard" siteId="{4a3d9983-e936-4837-9552-9d9126a92eb0}" contentBits="0" removed="0"/>

</xml_diff>